<commit_message>
12-12-2024 Update element and running background
</commit_message>
<xml_diff>
--- a/Excel/TC0001_LoginTravelio.xlsx
+++ b/Excel/TC0001_LoginTravelio.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\MetrocommJaddi\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\MetrocomJaddi\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75BC8394-0736-4604-B0BE-28830CF927FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231C7C01-CB9F-4AB5-B706-DA843046F3FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2F15E9A0-1C50-4655-9A11-8F4BEDD34A56}"/>
   </bookViews>
@@ -465,8 +465,8 @@
     <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="0.5703125" customWidth="1"/>
+    <col min="6" max="6" width="16" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>